<commit_message>
Agrega modal de confirmacion CONFIRMAR REGISTRO, botones REGISTRAR/CANCELAR, y delimitador de comas en datos.csv
Co-authored-by: muni26 <196358894+muni26@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mcal Lopex\Downloads\MUNI26\AA 30 07 MODIF\candidato 02 08\candidato-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE96EEC-EDA8-4D04-8CEF-B75411248873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6092D27B-42C1-4AED-8AD7-EEA18E31CD01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="datos" sheetId="2" r:id="rId1"/>
+    <sheet name="datos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,21 +25,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>cedula</t>
   </si>
   <si>
     <t>nro</t>
   </si>
-  <si>
-    <t>0992776729</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -71,9 +71,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -353,33 +351,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42F462EA-B910-4374-8ECF-3D03964C063E}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1477528</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
+      <c r="E1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="B2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>